<commit_message>
feat: add raw input columns to DOT/IOT/Invoice Conformity/Price Divergence KPI tables and update scorecard guide to 9 KPIs
</commit_message>
<xml_diff>
--- a/backend/feedback/uat_feedback.xlsx
+++ b/backend/feedback/uat_feedback.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,20 +424,25 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>page</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>username</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>comment</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>createdAt</t>
         </is>
@@ -446,25 +451,58 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>705c0fc6-087e-42f1-a52c-9f6ea38bdc86</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>scorecard</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Naren</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Check the logics</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-07-24T16:26:12.968531</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>25d67c15-eb08-4e39-bd46-ac800b8f6216</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
         <is>
           <t>Sarthak</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Improved UI</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>2026-07-23T15:29:19.550357</t>
         </is>

</xml_diff>